<commit_message>
Ajouter 3eme essai avec les essais existants
</commit_message>
<xml_diff>
--- a/resultat/resultats_macronutriments.xlsx
+++ b/resultat/resultats_macronutriments.xlsx
@@ -384,7 +384,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25.65 ± 0.04c</t>
+          <t>25.65 ± 0.03c</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>23.29 ± 0.04b</t>
+          <t>23.29 ± 0.03b</t>
         </is>
       </c>
     </row>
@@ -406,17 +406,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.87 ± 0.14b</t>
+          <t>0.87 ± 0.1b</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.29 ± 0.04a</t>
+          <t>1.28 ± 0.03a</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.98 ± 0.01ab</t>
+          <t>0.97 ± 0.01b</t>
         </is>
       </c>
     </row>
@@ -428,17 +428,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3.65 ± 0.18b</t>
+          <t>3.65 ± 0.13c</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.31 ± 0.21a</t>
+          <t>2.3 ± 0.15a</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.16 ± 0.08b</t>
+          <t>3.16 ± 0.06b</t>
         </is>
       </c>
     </row>
@@ -450,12 +450,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9.53 ± 0.15c</t>
+          <t>9.52 ± 0.11c</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>11.96 ± 0.13a</t>
+          <t>11.96 ± 0.09a</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -472,17 +472,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>60.3 ± 0.07c</t>
+          <t>60.3 ± 0.05c</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>58.64 ± 0.1a</t>
+          <t>58.64 ± 0.07a</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>62.67 ± 0.58b</t>
+          <t>62.67 ± 0.41b</t>
         </is>
       </c>
     </row>
@@ -494,17 +494,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>351.63 ± 0.82a</t>
+          <t>351.63 ± 0.58ab</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>349.36 ± 0.13a</t>
+          <t>349.36 ± 0.1a</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>352.55 ± 2.34a</t>
+          <t>352.55 ± 1.66b</t>
         </is>
       </c>
     </row>

</xml_diff>